<commit_message>
Modules 8A/8B completed & unit tested
</commit_message>
<xml_diff>
--- a/distillation_column_template.xlsx
+++ b/distillation_column_template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Thoma\Documents\Python Scripts\dynamic_distillation_GEKKO\AI Studio model\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Thoma\Documents\Python Scripts\Dynamic_DistillationII\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B18EE44-3F09-4191-8ACE-5A0AC1E29717}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1187D37-6697-4E3B-972D-66D2CE28F7BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="43">
   <si>
     <t>Parameter</t>
   </si>
@@ -148,6 +148,9 @@
   </si>
   <si>
     <t>Component 2</t>
+  </si>
+  <si>
+    <t>Stage time constant [tau] (sec)</t>
   </si>
 </sst>
 </file>
@@ -523,10 +526,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.42578125" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
     <col min="3" max="3" width="15.7109375" customWidth="1"/>
     <col min="4" max="4" width="13.7109375" customWidth="1"/>
@@ -627,6 +630,14 @@
       </c>
       <c r="B12">
         <v>100</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>42</v>
+      </c>
+      <c r="B13">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed Distillate Stream issue in the profile log.
</commit_message>
<xml_diff>
--- a/distillation_column_template.xlsx
+++ b/distillation_column_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Thoma\Documents\Python Scripts\Dynamic_DistillationII\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1455AE2-3608-4CF1-9490-790350470496}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{590719E5-1569-4388-BC05-0E486C6863B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -111,9 +111,6 @@
     <t xml:space="preserve">Feed </t>
   </si>
   <si>
-    <t xml:space="preserve">Top </t>
-  </si>
-  <si>
     <t xml:space="preserve">Bottom </t>
   </si>
   <si>
@@ -178,6 +175,9 @@
   </si>
   <si>
     <t>Active Area Fraction</t>
+  </si>
+  <si>
+    <t>Distillate</t>
   </si>
 </sst>
 </file>
@@ -604,7 +604,7 @@
         <v>6</v>
       </c>
       <c r="C5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D5" t="s">
         <v>7</v>
@@ -642,7 +642,7 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B10">
         <v>10</v>
@@ -650,7 +650,7 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B11">
         <v>0.1</v>
@@ -658,7 +658,7 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B12">
         <v>100</v>
@@ -666,7 +666,7 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B13">
         <v>10</v>
@@ -674,31 +674,31 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>47</v>
+      </c>
+      <c r="B15" t="s">
+        <v>42</v>
+      </c>
+      <c r="C15" t="s">
+        <v>43</v>
+      </c>
+      <c r="D15" t="s">
+        <v>44</v>
+      </c>
+      <c r="E15" t="s">
+        <v>45</v>
+      </c>
+      <c r="F15" t="s">
+        <v>46</v>
+      </c>
+      <c r="G15" t="s">
         <v>48</v>
       </c>
-      <c r="B15" t="s">
-        <v>43</v>
-      </c>
-      <c r="C15" t="s">
-        <v>44</v>
-      </c>
-      <c r="D15" t="s">
-        <v>45</v>
-      </c>
-      <c r="E15" t="s">
-        <v>46</v>
-      </c>
-      <c r="F15" t="s">
-        <v>47</v>
-      </c>
-      <c r="G15" t="s">
+      <c r="H15" t="s">
         <v>49</v>
       </c>
-      <c r="H15" t="s">
+      <c r="I15" t="s">
         <v>50</v>
-      </c>
-      <c r="I15" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -741,7 +741,7 @@
         <v>1.5</v>
       </c>
       <c r="F17">
-        <v>75</v>
+        <v>0.75</v>
       </c>
       <c r="G17">
         <v>2</v>
@@ -1675,15 +1675,15 @@
         <v>28</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B3">
         <v>12</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B4">
         <v>232.06</v>
@@ -1711,7 +1711,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -1725,7 +1725,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B6">
         <v>77</v>
@@ -1739,7 +1739,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B7">
         <v>7142.98</v>
@@ -1753,7 +1753,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -1786,7 +1786,7 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B12">
         <v>793.66399999999999</v>

</xml_diff>

<commit_message>
Snapshot: reboiler stage 20 and log updates
</commit_message>
<xml_diff>
--- a/distillation_column_template.xlsx
+++ b/distillation_column_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Thoma\Documents\Python Scripts\Dynamic_DistillationII\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{590719E5-1569-4388-BC05-0E486C6863B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E404AE4-8AC4-46E7-93C1-931E3F902DA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Specifications" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="54">
   <si>
     <t>Parameter</t>
   </si>
@@ -178,6 +178,12 @@
   </si>
   <si>
     <t>Distillate</t>
+  </si>
+  <si>
+    <t>Top Accumulator Holdup (lbmol)</t>
+  </si>
+  <si>
+    <t>Bottom Holdup (lbmol)</t>
   </si>
 </sst>
 </file>
@@ -553,10 +559,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="28.42578125" customWidth="1"/>
+    <col min="1" max="1" width="35.5703125" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
     <col min="3" max="3" width="15.7109375" customWidth="1"/>
     <col min="4" max="4" width="13.7109375" customWidth="1"/>
@@ -567,7 +573,7 @@
     <col min="9" max="9" width="17.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -575,7 +581,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -583,7 +589,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -591,7 +597,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -599,7 +605,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>6</v>
       </c>
@@ -610,7 +616,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -624,7 +630,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -632,7 +638,7 @@
         <v>-48500000</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -640,7 +646,7 @@
         <v>79124000</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>37</v>
       </c>
@@ -648,7 +654,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>38</v>
       </c>
@@ -656,7 +662,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>39</v>
       </c>
@@ -664,7 +670,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>41</v>
       </c>
@@ -672,84 +678,100 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>52</v>
+      </c>
+      <c r="B14">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>53</v>
+      </c>
+      <c r="B15">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>47</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B17" t="s">
         <v>42</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C17" t="s">
         <v>43</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D17" t="s">
         <v>44</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E17" t="s">
         <v>45</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F17" t="s">
         <v>46</v>
       </c>
-      <c r="G15" t="s">
+      <c r="G17" t="s">
         <v>48</v>
       </c>
-      <c r="H15" t="s">
+      <c r="H17" t="s">
         <v>49</v>
       </c>
-      <c r="I15" t="s">
+      <c r="I17" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B16">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B18">
         <v>2</v>
       </c>
-      <c r="C16">
+      <c r="C18">
         <v>15</v>
       </c>
-      <c r="D16">
+      <c r="D18">
         <v>16.9619</v>
       </c>
-      <c r="E16">
+      <c r="E18">
         <v>1.5</v>
       </c>
-      <c r="F16">
+      <c r="F18">
         <v>0.75</v>
       </c>
-      <c r="G16">
+      <c r="G18">
         <v>2</v>
       </c>
-      <c r="H16">
+      <c r="H18">
         <v>10</v>
       </c>
-      <c r="I16">
+      <c r="I18">
         <v>0.75</v>
       </c>
     </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B17">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B19">
         <v>16</v>
       </c>
-      <c r="C17">
+      <c r="C19">
         <v>20</v>
       </c>
-      <c r="D17">
+      <c r="D19">
         <v>18.175899999999999</v>
       </c>
-      <c r="E17">
+      <c r="E19">
         <v>1.5</v>
       </c>
-      <c r="F17">
+      <c r="F19">
         <v>0.75</v>
       </c>
-      <c r="G17">
+      <c r="G19">
         <v>2</v>
       </c>
-      <c r="H17">
+      <c r="H19">
         <v>9</v>
       </c>
-      <c r="I17">
+      <c r="I19">
         <v>0.75</v>
       </c>
     </row>
@@ -832,7 +854,7 @@
         <v>5952.48</v>
       </c>
       <c r="F2">
-        <v>992</v>
+        <v>0</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -1629,7 +1651,7 @@
         <v>0</v>
       </c>
       <c r="F21">
-        <v>694</v>
+        <v>0</v>
       </c>
       <c r="G21">
         <v>10</v>

</xml_diff>

<commit_message>
Include updated distillation column template workbook
</commit_message>
<xml_diff>
--- a/distillation_column_template.xlsx
+++ b/distillation_column_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Thoma\Documents\Python Scripts\Dynamic_DistillationII\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73EB3BCC-ECB4-442B-92C8-A2438B94BD63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55D9EA3E-022C-4093-852F-52556AE8D1E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,12 +17,12 @@
     <sheet name="Initial Conditions" sheetId="2" r:id="rId2"/>
     <sheet name="Streams" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="65">
   <si>
     <t>Parameter</t>
   </si>
@@ -45,6 +45,9 @@
     <t>Component 1</t>
   </si>
   <si>
+    <t>Component 2</t>
+  </si>
+  <si>
     <t>Component 3</t>
   </si>
   <si>
@@ -66,6 +69,87 @@
     <t>Reboiler Duty (Btu/h)</t>
   </si>
   <si>
+    <t>Simulation Length (min)</t>
+  </si>
+  <si>
+    <t>Timestep (sec)</t>
+  </si>
+  <si>
+    <t>Log Frequency (timesteps)</t>
+  </si>
+  <si>
+    <t>Thermo refresh Delta T (F)</t>
+  </si>
+  <si>
+    <t>Stage time constant [tau] (sec)</t>
+  </si>
+  <si>
+    <t>Top Accumulator Holdup (lbmol)</t>
+  </si>
+  <si>
+    <t>Bottom Holdup (lbmol)</t>
+  </si>
+  <si>
+    <t>Vapor Holdup Relaxation (sec)</t>
+  </si>
+  <si>
+    <t>Vapor Flow Relaxation (sec) </t>
+  </si>
+  <si>
+    <t>Dry Tray K</t>
+  </si>
+  <si>
+    <t>Pressure Model</t>
+  </si>
+  <si>
+    <t>Hydraulic</t>
+  </si>
+  <si>
+    <t>Vapor Flow Model</t>
+  </si>
+  <si>
+    <t>energy</t>
+  </si>
+  <si>
+    <t>Condenser Pressure Drop (psi)</t>
+  </si>
+  <si>
+    <t>Distillate Drum Diameter (ft)</t>
+  </si>
+  <si>
+    <t>Distillate Drum Length (ft)</t>
+  </si>
+  <si>
+    <t>Distillate Drum Liquid Fraction</t>
+  </si>
+  <si>
+    <t>Stage Geometry</t>
+  </si>
+  <si>
+    <t>Start Stage</t>
+  </si>
+  <si>
+    <t>End Stage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diameter (ft) </t>
+  </si>
+  <si>
+    <t>Tray Spacing (ft)</t>
+  </si>
+  <si>
+    <t>Gas Void Fraction</t>
+  </si>
+  <si>
+    <t>Weir Height (in)</t>
+  </si>
+  <si>
+    <t>Weir Length (ft)</t>
+  </si>
+  <si>
+    <t>Active Area Fraction</t>
+  </si>
+  <si>
     <t>Stage</t>
   </si>
   <si>
@@ -84,9 +168,6 @@
     <t>Liquid Holdup (lbmol)</t>
   </si>
   <si>
-    <t>Vapor Holdup (lbmol)</t>
-  </si>
-  <si>
     <t>Vapor Composition Component 1</t>
   </si>
   <si>
@@ -111,6 +192,9 @@
     <t xml:space="preserve">Feed </t>
   </si>
   <si>
+    <t>Distillate</t>
+  </si>
+  <si>
     <t xml:space="preserve">Bottom </t>
   </si>
   <si>
@@ -133,57 +217,6 @@
   </si>
   <si>
     <t>N-Pentane</t>
-  </si>
-  <si>
-    <t>Simulation Length (min)</t>
-  </si>
-  <si>
-    <t>Timestep (sec)</t>
-  </si>
-  <si>
-    <t>Log Frequency (timesteps)</t>
-  </si>
-  <si>
-    <t>Component 2</t>
-  </si>
-  <si>
-    <t>Stage time constant [tau] (sec)</t>
-  </si>
-  <si>
-    <t>Start Stage</t>
-  </si>
-  <si>
-    <t>End Stage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Diameter (ft) </t>
-  </si>
-  <si>
-    <t>Tray Spacing (ft)</t>
-  </si>
-  <si>
-    <t>Gas Void Fraction</t>
-  </si>
-  <si>
-    <t>Stage Geometry</t>
-  </si>
-  <si>
-    <t>Weir Height (in)</t>
-  </si>
-  <si>
-    <t>Weir Length (ft)</t>
-  </si>
-  <si>
-    <t>Active Area Fraction</t>
-  </si>
-  <si>
-    <t>Distillate</t>
-  </si>
-  <si>
-    <t>Top Accumulator Holdup (lbmol)</t>
-  </si>
-  <si>
-    <t>Bottom Holdup (lbmol)</t>
   </si>
 </sst>
 </file>
@@ -559,7 +592,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.5703125" customWidth="1"/>
@@ -610,29 +643,29 @@
         <v>6</v>
       </c>
       <c r="C5" t="s">
-        <v>40</v>
+        <v>7</v>
       </c>
       <c r="D5" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B7">
         <v>-48500000</v>
@@ -640,7 +673,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B8">
         <v>79124000</v>
@@ -648,15 +681,15 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="B10">
-        <v>0.16667000000000001</v>
+        <v>6.6666599999999996E-3</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="B11">
         <v>0.2</v>
@@ -664,114 +697,217 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="B12">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>41</v>
-      </c>
-      <c r="B13">
-        <v>10</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>52</v>
+        <v>19</v>
       </c>
       <c r="B14">
-        <v>397</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>53</v>
+        <v>20</v>
       </c>
       <c r="B15">
+        <v>1388.9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16">
         <v>794</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>47</v>
-      </c>
-      <c r="B17" t="s">
-        <v>42</v>
-      </c>
-      <c r="C17" t="s">
-        <v>43</v>
-      </c>
-      <c r="D17" t="s">
-        <v>44</v>
-      </c>
-      <c r="E17" t="s">
-        <v>45</v>
-      </c>
-      <c r="F17" t="s">
-        <v>46</v>
-      </c>
-      <c r="G17" t="s">
-        <v>48</v>
-      </c>
-      <c r="H17" t="s">
-        <v>49</v>
-      </c>
-      <c r="I17" t="s">
-        <v>50</v>
+        <v>22</v>
+      </c>
+      <c r="B17">
+        <v>25</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>23</v>
+      </c>
       <c r="B18">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>24</v>
+      </c>
+      <c r="B19">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>25</v>
+      </c>
+      <c r="B20" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>27</v>
+      </c>
+      <c r="B21" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>29</v>
+      </c>
+      <c r="B22">
         <v>2</v>
       </c>
-      <c r="C18">
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>30</v>
+      </c>
+      <c r="B24">
+        <v>12.1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>31</v>
+      </c>
+      <c r="B25">
+        <v>36.299999999999997</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>32</v>
+      </c>
+      <c r="B26">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>33</v>
+      </c>
+      <c r="B28" t="s">
+        <v>34</v>
+      </c>
+      <c r="C28" t="s">
+        <v>35</v>
+      </c>
+      <c r="D28" t="s">
+        <v>36</v>
+      </c>
+      <c r="E28" t="s">
+        <v>37</v>
+      </c>
+      <c r="F28" t="s">
+        <v>38</v>
+      </c>
+      <c r="G28" t="s">
+        <v>39</v>
+      </c>
+      <c r="H28" t="s">
+        <v>40</v>
+      </c>
+      <c r="I28" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B29">
+        <v>2</v>
+      </c>
+      <c r="C29">
+        <v>2</v>
+      </c>
+      <c r="D29">
+        <v>16.9619</v>
+      </c>
+      <c r="E29">
+        <v>5</v>
+      </c>
+      <c r="F29">
+        <v>0.75</v>
+      </c>
+      <c r="G29">
+        <v>2</v>
+      </c>
+      <c r="H29">
+        <v>9</v>
+      </c>
+      <c r="I29">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B30">
+        <v>3</v>
+      </c>
+      <c r="C30">
         <v>15</v>
       </c>
-      <c r="D18">
+      <c r="D30">
         <v>16.9619</v>
       </c>
-      <c r="E18">
+      <c r="E30">
         <v>1.5</v>
       </c>
-      <c r="F18">
+      <c r="F30">
         <v>0.75</v>
       </c>
-      <c r="G18">
+      <c r="G30">
         <v>2</v>
       </c>
-      <c r="H18">
+      <c r="H30">
+        <v>9</v>
+      </c>
+      <c r="I30">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B31">
+        <v>16</v>
+      </c>
+      <c r="C31">
+        <v>20</v>
+      </c>
+      <c r="D31">
+        <v>18.175899999999999</v>
+      </c>
+      <c r="E31">
+        <v>1.5</v>
+      </c>
+      <c r="F31">
+        <v>0.75</v>
+      </c>
+      <c r="G31">
+        <v>2</v>
+      </c>
+      <c r="H31">
         <v>10</v>
       </c>
-      <c r="I18">
-        <v>0.75</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B19">
-        <v>16</v>
-      </c>
-      <c r="C19">
-        <v>20</v>
-      </c>
-      <c r="D19">
-        <v>18.175899999999999</v>
-      </c>
-      <c r="E19">
-        <v>1.5</v>
-      </c>
-      <c r="F19">
-        <v>0.75</v>
-      </c>
-      <c r="G19">
-        <v>2</v>
-      </c>
-      <c r="H19">
-        <v>9</v>
-      </c>
-      <c r="I19">
+      <c r="I31">
         <v>0.75</v>
       </c>
     </row>
@@ -782,7 +918,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:M21"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr defaultColWidth="34.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.85546875" bestFit="1" customWidth="1"/>
@@ -791,53 +927,49 @@
     <col min="4" max="4" width="20.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="10" width="31" bestFit="1" customWidth="1"/>
-    <col min="11" max="13" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="31" bestFit="1" customWidth="1"/>
+    <col min="10" max="12" width="31.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>14</v>
+        <v>42</v>
       </c>
       <c r="B1" t="s">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>16</v>
+        <v>44</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>17</v>
+        <v>45</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>18</v>
+        <v>46</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>19</v>
+        <v>47</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>20</v>
+        <v>48</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>21</v>
+        <v>49</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>22</v>
+        <v>50</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>24</v>
+        <v>52</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -845,7 +977,7 @@
         <v>115.556</v>
       </c>
       <c r="C2">
-        <v>219.44</v>
+        <v>218.44</v>
       </c>
       <c r="D2">
         <v>0</v>
@@ -857,28 +989,25 @@
         <v>0</v>
       </c>
       <c r="G2">
-        <v>0</v>
+        <v>0.97869099999999998</v>
       </c>
       <c r="H2">
-        <v>0.97869099999999998</v>
+        <v>2.13086E-2</v>
       </c>
       <c r="I2">
-        <v>2.13086E-2</v>
+        <v>3.094E-7</v>
       </c>
       <c r="J2">
-        <v>3.094E-7</v>
+        <v>0.94906000000000001</v>
       </c>
       <c r="K2">
-        <v>0.94906000000000001</v>
+        <v>5.0938299999999999E-2</v>
       </c>
       <c r="L2">
-        <v>5.0938299999999999E-2</v>
-      </c>
-      <c r="M2">
         <v>1.7689999999999999E-6</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -898,28 +1027,25 @@
         <v>33.1</v>
       </c>
       <c r="G3">
-        <v>9</v>
+        <v>0.94906000000000001</v>
       </c>
       <c r="H3">
-        <v>0.94906000000000001</v>
+        <v>5.0938299999999999E-2</v>
       </c>
       <c r="I3">
-        <v>5.0938299999999999E-2</v>
+        <v>1.7689999999999999E-6</v>
       </c>
       <c r="J3">
-        <v>1.7689999999999999E-6</v>
+        <v>0.88409199999999999</v>
       </c>
       <c r="K3">
-        <v>0.88409199999999999</v>
+        <v>0.115899</v>
       </c>
       <c r="L3">
-        <v>0.115899</v>
-      </c>
-      <c r="M3">
         <v>9.5363000000000005E-6</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -939,28 +1065,25 @@
         <v>32.6</v>
       </c>
       <c r="G4">
-        <v>9</v>
+        <v>0.90310699999999999</v>
       </c>
       <c r="H4">
-        <v>0.90310699999999999</v>
+        <v>9.6885700000000005E-2</v>
       </c>
       <c r="I4">
-        <v>9.6885700000000005E-2</v>
+        <v>7.2629999999999997E-6</v>
       </c>
       <c r="J4">
-        <v>7.2629999999999997E-6</v>
+        <v>0.79485499999999998</v>
       </c>
       <c r="K4">
-        <v>0.79485499999999998</v>
+        <v>0.20510900000000001</v>
       </c>
       <c r="L4">
-        <v>0.20510900000000001</v>
-      </c>
-      <c r="M4">
         <v>3.5868000000000003E-5</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -980,28 +1103,25 @@
         <v>32.200000000000003</v>
       </c>
       <c r="G5">
-        <v>9</v>
+        <v>0.84120300000000003</v>
       </c>
       <c r="H5">
-        <v>0.84120300000000003</v>
+        <v>0.158771</v>
       </c>
       <c r="I5">
-        <v>0.158771</v>
+        <v>2.5619E-5</v>
       </c>
       <c r="J5">
-        <v>2.5619E-5</v>
+        <v>0.69183499999999998</v>
       </c>
       <c r="K5">
-        <v>0.69183499999999998</v>
+        <v>0.30805100000000002</v>
       </c>
       <c r="L5">
-        <v>0.30805100000000002</v>
-      </c>
-      <c r="M5">
         <v>1.1370999999999999E-4</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1021,28 +1141,25 @@
         <v>31.9</v>
       </c>
       <c r="G6">
-        <v>9</v>
+        <v>0.77103299999999997</v>
       </c>
       <c r="H6">
-        <v>0.77103299999999997</v>
+        <v>0.22888800000000001</v>
       </c>
       <c r="I6">
-        <v>0.22888800000000001</v>
+        <v>7.9249E-5</v>
       </c>
       <c r="J6">
-        <v>7.9249E-5</v>
+        <v>0.59292800000000001</v>
       </c>
       <c r="K6">
-        <v>0.59292800000000001</v>
+        <v>0.40675600000000001</v>
       </c>
       <c r="L6">
-        <v>0.40675600000000001</v>
-      </c>
-      <c r="M6">
         <v>3.1562000000000002E-4</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1062,28 +1179,25 @@
         <v>31.8</v>
       </c>
       <c r="G7">
-        <v>9</v>
+        <v>0.70448599999999995</v>
       </c>
       <c r="H7">
-        <v>0.70448599999999995</v>
+        <v>0.29529699999999998</v>
       </c>
       <c r="I7">
-        <v>0.29529699999999998</v>
+        <v>2.173E-4</v>
       </c>
       <c r="J7">
-        <v>2.173E-4</v>
+        <v>0.51219400000000004</v>
       </c>
       <c r="K7">
-        <v>0.51219400000000004</v>
+        <v>0.48701800000000001</v>
       </c>
       <c r="L7">
-        <v>0.48701800000000001</v>
-      </c>
-      <c r="M7">
         <v>7.8854999999999995E-4</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1103,28 +1217,25 @@
         <v>31.7</v>
       </c>
       <c r="G8">
-        <v>9</v>
+        <v>0.65042800000000001</v>
       </c>
       <c r="H8">
-        <v>0.65042800000000001</v>
+        <v>0.34903299999999998</v>
       </c>
       <c r="I8">
-        <v>0.34903299999999998</v>
+        <v>5.396E-4</v>
       </c>
       <c r="J8">
-        <v>5.396E-4</v>
+        <v>0.45379599999999998</v>
       </c>
       <c r="K8">
-        <v>0.45379599999999998</v>
+        <v>0.54437899999999995</v>
       </c>
       <c r="L8">
-        <v>0.54437899999999995</v>
-      </c>
-      <c r="M8">
         <v>1.8251700000000001E-3</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1144,28 +1255,25 @@
         <v>31.6</v>
       </c>
       <c r="G9">
-        <v>9</v>
+        <v>0.61133599999999999</v>
       </c>
       <c r="H9">
-        <v>0.61133599999999999</v>
+        <v>0.38741900000000001</v>
       </c>
       <c r="I9">
-        <v>0.38741900000000001</v>
+        <v>1.2451599999999999E-3</v>
       </c>
       <c r="J9">
-        <v>1.2451599999999999E-3</v>
+        <v>0.41470600000000002</v>
       </c>
       <c r="K9">
-        <v>0.41470600000000002</v>
+        <v>0.58128400000000002</v>
       </c>
       <c r="L9">
-        <v>0.58128400000000002</v>
-      </c>
-      <c r="M9">
         <v>4.0092799999999996E-3</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1185,28 +1293,25 @@
         <v>31.6</v>
       </c>
       <c r="G10">
-        <v>9</v>
+        <v>0.585202</v>
       </c>
       <c r="H10">
-        <v>0.585202</v>
+        <v>0.41206799999999999</v>
       </c>
       <c r="I10">
-        <v>0.41206799999999999</v>
+        <v>2.7306100000000001E-3</v>
       </c>
       <c r="J10">
-        <v>2.7306100000000001E-3</v>
+        <v>0.38949499999999998</v>
       </c>
       <c r="K10">
-        <v>0.38949499999999998</v>
+        <v>0.60200799999999999</v>
       </c>
       <c r="L10">
-        <v>0.60200799999999999</v>
-      </c>
-      <c r="M10">
         <v>8.4970299999999992E-3</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1226,28 +1331,25 @@
         <v>31.5</v>
       </c>
       <c r="G11">
-        <v>8</v>
+        <v>0.56855199999999995</v>
       </c>
       <c r="H11">
-        <v>0.56855199999999995</v>
+        <v>0.42566999999999999</v>
       </c>
       <c r="I11">
-        <v>0.42566999999999999</v>
+        <v>5.77861E-3</v>
       </c>
       <c r="J11">
-        <v>5.77861E-3</v>
+        <v>0.37301299999999998</v>
       </c>
       <c r="K11">
-        <v>0.37301299999999998</v>
+        <v>0.60946500000000003</v>
       </c>
       <c r="L11">
-        <v>0.60946500000000003</v>
-      </c>
-      <c r="M11">
         <v>1.7522200000000002E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1267,28 +1369,25 @@
         <v>31.4</v>
       </c>
       <c r="G12">
-        <v>8</v>
+        <v>0.55818699999999999</v>
       </c>
       <c r="H12">
-        <v>0.55818699999999999</v>
+        <v>0.429923</v>
       </c>
       <c r="I12">
-        <v>0.429923</v>
+        <v>1.1890100000000001E-2</v>
       </c>
       <c r="J12">
-        <v>1.1890100000000001E-2</v>
+        <v>0.36106100000000002</v>
       </c>
       <c r="K12">
-        <v>0.36106100000000002</v>
+        <v>0.60375800000000002</v>
       </c>
       <c r="L12">
-        <v>0.60375800000000002</v>
-      </c>
-      <c r="M12">
         <v>3.5180900000000001E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1308,28 +1407,25 @@
         <v>50.6</v>
       </c>
       <c r="G13">
-        <v>6</v>
+        <v>0.55166700000000002</v>
       </c>
       <c r="H13">
-        <v>0.55166700000000002</v>
+        <v>0.42455599999999999</v>
       </c>
       <c r="I13">
-        <v>0.42455599999999999</v>
+        <v>2.3777199999999998E-2</v>
       </c>
       <c r="J13">
-        <v>2.3777199999999998E-2</v>
+        <v>0.350163</v>
       </c>
       <c r="K13">
-        <v>0.350163</v>
+        <v>0.58161300000000005</v>
       </c>
       <c r="L13">
-        <v>0.58161300000000005</v>
-      </c>
-      <c r="M13">
         <v>6.8223699999999998E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1349,28 +1445,25 @@
         <v>50.7</v>
       </c>
       <c r="G14">
-        <v>10</v>
+        <v>0.48916999999999999</v>
       </c>
       <c r="H14">
-        <v>0.48916999999999999</v>
+        <v>0.48475099999999999</v>
       </c>
       <c r="I14">
-        <v>0.48475099999999999</v>
+        <v>2.60792E-2</v>
       </c>
       <c r="J14">
-        <v>2.60792E-2</v>
+        <v>0.29932399999999998</v>
       </c>
       <c r="K14">
-        <v>0.29932399999999998</v>
+        <v>0.63065099999999996</v>
       </c>
       <c r="L14">
-        <v>0.63065099999999996</v>
-      </c>
-      <c r="M14">
         <v>7.0025000000000004E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1390,28 +1483,25 @@
         <v>50.8</v>
       </c>
       <c r="G15">
-        <v>10</v>
+        <v>0.416184</v>
       </c>
       <c r="H15">
-        <v>0.416184</v>
+        <v>0.55503000000000002</v>
       </c>
       <c r="I15">
-        <v>0.55503000000000002</v>
+        <v>2.8786099999999998E-2</v>
       </c>
       <c r="J15">
-        <v>2.8786099999999998E-2</v>
+        <v>0.244946</v>
       </c>
       <c r="K15">
-        <v>0.244946</v>
+        <v>0.68310899999999997</v>
       </c>
       <c r="L15">
-        <v>0.68310899999999997</v>
-      </c>
-      <c r="M15">
         <v>7.1945499999999996E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1431,28 +1521,25 @@
         <v>51</v>
       </c>
       <c r="G16">
-        <v>10</v>
+        <v>0.33793200000000001</v>
       </c>
       <c r="H16">
-        <v>0.33793200000000001</v>
+        <v>0.63025299999999995</v>
       </c>
       <c r="I16">
-        <v>0.63025299999999995</v>
+        <v>3.18149E-2</v>
       </c>
       <c r="J16">
-        <v>3.18149E-2</v>
+        <v>0.191524</v>
       </c>
       <c r="K16">
-        <v>0.191524</v>
+        <v>0.73442499999999999</v>
       </c>
       <c r="L16">
-        <v>0.73442499999999999</v>
-      </c>
-      <c r="M16">
         <v>7.4051599999999995E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1472,28 +1559,25 @@
         <v>61.8</v>
       </c>
       <c r="G17">
-        <v>10</v>
+        <v>0.26112099999999999</v>
       </c>
       <c r="H17">
-        <v>0.26112099999999999</v>
+        <v>0.70364400000000005</v>
       </c>
       <c r="I17">
-        <v>0.70364400000000005</v>
+        <v>3.5234500000000002E-2</v>
       </c>
       <c r="J17">
-        <v>3.5234500000000002E-2</v>
+        <v>0.14307500000000001</v>
       </c>
       <c r="K17">
-        <v>0.14307500000000001</v>
+        <v>0.78010800000000002</v>
       </c>
       <c r="L17">
-        <v>0.78010800000000002</v>
-      </c>
-      <c r="M17">
         <v>7.6816700000000002E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1513,28 +1597,25 @@
         <v>62.1</v>
       </c>
       <c r="G18">
-        <v>9.5</v>
+        <v>0.19173999999999999</v>
       </c>
       <c r="H18">
-        <v>0.19173999999999999</v>
+        <v>0.76862299999999995</v>
       </c>
       <c r="I18">
-        <v>0.76862299999999995</v>
+        <v>3.9636999999999999E-2</v>
       </c>
       <c r="J18">
-        <v>3.9636999999999999E-2</v>
+        <v>0.102089</v>
       </c>
       <c r="K18">
-        <v>0.102089</v>
+        <v>0.81628000000000001</v>
       </c>
       <c r="L18">
-        <v>0.81628000000000001</v>
-      </c>
-      <c r="M18">
         <v>8.1630499999999995E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1554,28 +1635,25 @@
         <v>62.2</v>
       </c>
       <c r="G19">
-        <v>9.5</v>
+        <v>0.133411</v>
       </c>
       <c r="H19">
-        <v>0.133411</v>
+        <v>0.81972100000000003</v>
       </c>
       <c r="I19">
-        <v>0.81972100000000003</v>
+        <v>4.6868399999999998E-2</v>
       </c>
       <c r="J19">
-        <v>4.6868399999999998E-2</v>
+        <v>6.93082E-2</v>
       </c>
       <c r="K19">
-        <v>6.93082E-2</v>
+        <v>0.83881700000000003</v>
       </c>
       <c r="L19">
-        <v>0.83881700000000003</v>
-      </c>
-      <c r="M19">
         <v>9.1874499999999998E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1595,28 +1673,25 @@
         <v>62.2</v>
       </c>
       <c r="G20">
-        <v>9</v>
+        <v>8.7082300000000001E-2</v>
       </c>
       <c r="H20">
-        <v>8.7082300000000001E-2</v>
+        <v>0.85136699999999998</v>
       </c>
       <c r="I20">
-        <v>0.85136699999999998</v>
+        <v>6.1550399999999998E-2</v>
       </c>
       <c r="J20">
-        <v>6.1550399999999998E-2</v>
+        <v>4.4168699999999998E-2</v>
       </c>
       <c r="K20">
-        <v>4.4168699999999998E-2</v>
+        <v>0.84071600000000002</v>
       </c>
       <c r="L20">
-        <v>0.84071600000000002</v>
-      </c>
-      <c r="M20">
         <v>0.115116</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1636,24 +1711,21 @@
         <v>0</v>
       </c>
       <c r="G21">
-        <v>10</v>
+        <v>5.1750900000000002E-2</v>
       </c>
       <c r="H21">
-        <v>5.1750900000000002E-2</v>
+        <v>0.85403700000000005</v>
       </c>
       <c r="I21">
-        <v>0.85403700000000005</v>
+        <v>9.4212000000000004E-2</v>
       </c>
       <c r="J21">
-        <v>9.4212000000000004E-2</v>
+        <v>2.547E-2</v>
       </c>
       <c r="K21">
-        <v>2.547E-2</v>
+        <v>0.80786400000000003</v>
       </c>
       <c r="L21">
-        <v>0.80786400000000003</v>
-      </c>
-      <c r="M21">
         <v>0.16666600000000001</v>
       </c>
     </row>
@@ -1673,21 +1745,21 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>27</v>
+        <v>54</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>28</v>
+        <v>55</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>29</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>30</v>
+        <v>58</v>
       </c>
       <c r="B3">
         <v>12</v>
@@ -1701,13 +1773,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>31</v>
+        <v>59</v>
       </c>
       <c r="B4">
         <v>232.06</v>
       </c>
       <c r="C4">
-        <v>220.44</v>
+        <v>218.44</v>
       </c>
       <c r="D4">
         <v>232.06</v>
@@ -1715,7 +1787,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>32</v>
+        <v>60</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -1729,7 +1801,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>33</v>
+        <v>61</v>
       </c>
       <c r="B6">
         <v>77</v>
@@ -1743,7 +1815,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>34</v>
+        <v>62</v>
       </c>
       <c r="B7">
         <v>7142.98</v>
@@ -1757,12 +1829,12 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>35</v>
+        <v>63</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B10">
         <v>2380.9899999999998</v>
@@ -1776,7 +1848,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B11">
         <v>3968.32</v>
@@ -1790,7 +1862,7 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>36</v>
+        <v>64</v>
       </c>
       <c r="B12">
         <v>793.66399999999999</v>

</xml_diff>